<commit_message>
fix(div7a-loan-review): flag fabricated example loans left in the workbook register
A Sample_row column matches the shipped loan_id and year pairs and Review
Checks returns REVIEW while any remains, so a register pasted over fewer
rows than the example cannot carry sample loans into the summary. Rules
changed: none.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC695714-6E02-41E0-84D9-6326A54871BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCBBE89-F138-4682-889B-232CFE7A1EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="151">
   <si>
     <t>Division 7A loan review: s 109N terms and s 109E minimum yearly repayment</t>
   </si>
@@ -170,6 +170,9 @@
     <t>Input_problem</t>
   </si>
   <si>
+    <t>Sample_row</t>
+  </si>
+  <si>
     <t>L-101</t>
   </si>
   <si>
@@ -411,6 +414,9 @@
   </si>
   <si>
     <t>Rows refused a repayment figure (read the reason; not a breach by itself)</t>
+  </si>
+  <si>
+    <t>No fabricated example loan from the shipped sample remains in the register</t>
   </si>
   <si>
     <t>Caveats the engine attaches to every result</t>
@@ -667,8 +673,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblLoans" displayName="tblLoans" ref="A1:AI9">
-  <tableColumns count="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblLoans" displayName="tblLoans" ref="A1:AJ9">
+  <tableColumns count="36">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="loan_id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="borrower_reference"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="year_loan_made"/>
@@ -745,6 +751,9 @@
     </tableColumn>
     <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Input_problem">
       <calculatedColumnFormula>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Sample_row">
+      <calculatedColumnFormula>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1126,7 +1135,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AI9"/>
+  <dimension ref="A1:AJ9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1138,10 +1147,10 @@
     <col min="14" max="28" width="12" customWidth="1"/>
     <col min="29" max="29" width="40" customWidth="1"/>
     <col min="30" max="32" width="14" customWidth="1"/>
-    <col min="33" max="35" width="12" customWidth="1"/>
+    <col min="33" max="36" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>9</v>
       </c>
@@ -1247,31 +1256,34 @@
       <c r="AI1" s="5" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ1" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F2" s="7">
         <v>7</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I2" s="7">
         <v>8.2699999999999996E-2</v>
@@ -1371,31 +1383,35 @@
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
       </c>
-    </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ2" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F3" s="7">
         <v>7</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I3" s="7">
         <v>0.04</v>
@@ -1495,31 +1511,35 @@
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
       </c>
-    </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ3" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F4" s="7">
         <v>7</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I4" s="7">
         <v>4.5199999999999997E-2</v>
@@ -1619,31 +1639,35 @@
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
       </c>
-    </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ4" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F5" s="7">
         <v>7</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I5" s="7">
         <v>8.77E-2</v>
@@ -1655,7 +1679,7 @@
         <v>5</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
@@ -1743,31 +1767,35 @@
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
       </c>
-    </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ5" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F6" s="7">
         <v>7</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I6" s="7">
         <v>5.3699999999999998E-2</v>
@@ -1867,28 +1895,32 @@
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
       </c>
-    </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ6" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F7" s="7">
         <v>25</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H7" s="7">
         <v>1.0900000000000001</v>
@@ -1991,46 +2023,50 @@
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
       </c>
-    </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ7" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="L8" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N8" s="6"/>
       <c r="O8" s="9" t="str">
@@ -2117,31 +2153,35 @@
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
       </c>
-    </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ8" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F9" s="7">
         <v>7</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I9" s="7">
         <v>7.0000000000000007E-2</v>
@@ -2240,6 +2280,10 @@
       <c r="AI9" s="9" t="str">
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
+      </c>
+      <c r="AJ9" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2265,214 +2309,214 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" s="7">
         <v>5.3699999999999998E-2</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B3" s="7">
         <v>4.5199999999999997E-2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E3" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="G3" s="7" t="s">
         <v>83</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B4" s="7">
         <v>4.5199999999999997E-2</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B5" s="7">
         <v>4.7699999999999999E-2</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B6" s="7">
         <v>8.2699999999999996E-2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B7" s="7">
         <v>8.77E-2</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B8" s="7">
         <v>8.3699999999999997E-2</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B9" s="7">
         <v>8.77E-2</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -2494,21 +2538,21 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B1" s="5"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B3" s="12">
         <f>IFERROR(INDEX(tblRates[rate],MATCH(B2,tblRates[year_of_income],0)),"")</f>
@@ -2517,7 +2561,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B4" s="9">
         <f>IFERROR(VALUE(LEFT(B2,4)),"")</f>
@@ -2526,13 +2570,13 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B6" s="5"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B7" s="9">
         <f>COUNTIF(tblLoans[Status],"REVIEWED")</f>
@@ -2541,7 +2585,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B8" s="9">
         <f>COUNTIF(tblLoans[Gate_verdict],"COMPLYING")</f>
@@ -2550,7 +2594,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B9" s="9">
         <f>COUNTIF(tblLoans[Gate_verdict],"NOT_COMPLYING")</f>
@@ -2559,7 +2603,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B10" s="9">
         <f>COUNTIF(tblLoans[MYR_verdict],"MYR_MET")</f>
@@ -2568,7 +2612,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B11" s="9">
         <f>COUNTIF(tblLoans[MYR_verdict],"MYR_SHORT")</f>
@@ -2577,7 +2621,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B12" s="9">
         <f>SUM(tblLoans[Undecided])</f>
@@ -2586,7 +2630,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B13" s="9">
         <f>COUNTIF(tblLoans[MYR_verdict],"REFUSED")</f>
@@ -2595,7 +2639,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B14" s="9">
         <f>COUNTIF(tblLoans[Status],"SKIPPED")</f>
@@ -2604,7 +2648,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B15" s="10">
         <f>SUM(tblLoans[Exposure])</f>
@@ -2661,21 +2705,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B2" s="9" t="str">
         <f>IF(C2=0,"PASS","BLOCKED")</f>
@@ -2692,7 +2736,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B3" s="9" t="str">
         <f>IF(C3=0,"PASS","BLOCKED")</f>
@@ -2709,7 +2753,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B4" s="9" t="str">
         <f>IF(ISNUMBER(Summary!B3),"PASS","BLOCKED")</f>
@@ -2723,7 +2767,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B5" s="9" t="str">
         <f>IF(C5=0,"PASS","REVIEW")</f>
@@ -2740,7 +2784,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B6" s="9" t="str">
         <f>IF(C6=0,"PASS","REVIEW")</f>
@@ -2757,7 +2801,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B7" s="9" t="str">
         <f>IF(C7=0,"PASS","REVIEW")</f>
@@ -2774,7 +2818,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B8" s="9" t="str">
         <f>IF(C8=0,"PASS","NOTE")</f>
@@ -2789,43 +2833,60 @@
         <v>L-106</v>
       </c>
     </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B9" s="9" t="str">
+        <f>IF(C9=0,"PASS","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="C9" s="9">
+        <f>SUM(tblLoans[Sample_row])</f>
+        <v>8</v>
+      </c>
+      <c r="D9" s="9" t="str">
+        <f t="array" ref="D9">IF(C9=0,"",INDEX(tblLoans[loan_id],SUMPRODUCT(MAX((tblLoans[Sample_row]=1)*(ROW(tblLoans[loan_id])-1)))))</f>
+        <v>L-108</v>
+      </c>
+    </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="13" t="str">
-        <f>IF(COUNTIF(B2:B8,"BLOCKED")&gt;0,"BLOCKED",IF(COUNTIF(B2:B8,"REVIEW")&gt;0,"REVIEW","PASS"))</f>
+        <f>IF(COUNTIF(B2:B9,"BLOCKED")&gt;0,"BLOCKED",IF(COUNTIF(B2:B9,"REVIEW")&gt;0,"REVIEW","PASS"))</f>
         <v>REVIEW</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -2856,82 +2917,82 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B4" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B10" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(workbooks): flag fabricated example rows left in the ATO and Div 7A workbooks (#98)
* fix(ato-benchmark-compare): flag fabricated example lines left in the workbook P&L

A Sample column matches the shipped bakery account-and-amount pairs and
Review Checks returns REVIEW while any remains, so a register pasted over
fewer rows than the example cannot carry sample lines into the ratios.
Rules changed: none; the parity test now expects the sample at REVIEW.

* fix(div7a-loan-review): flag fabricated example loans left in the workbook register

A Sample_row column matches the shipped loan_id and year pairs and Review
Checks returns REVIEW while any remains, so a register pasted over fewer
rows than the example cannot carry sample loans into the summary. Rules
changed: none.
</commit_message>
<xml_diff>
--- a/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
+++ b/packages/div7a-loan-review/workbooks/div7a-loan-review.xlsx
@@ -6,7 +6,7 @@
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC695714-6E02-41E0-84D9-6326A54871BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCBBE89-F138-4682-889B-232CFE7A1EB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="151">
   <si>
     <t>Division 7A loan review: s 109N terms and s 109E minimum yearly repayment</t>
   </si>
@@ -170,6 +170,9 @@
     <t>Input_problem</t>
   </si>
   <si>
+    <t>Sample_row</t>
+  </si>
+  <si>
     <t>L-101</t>
   </si>
   <si>
@@ -411,6 +414,9 @@
   </si>
   <si>
     <t>Rows refused a repayment figure (read the reason; not a breach by itself)</t>
+  </si>
+  <si>
+    <t>No fabricated example loan from the shipped sample remains in the register</t>
   </si>
   <si>
     <t>Caveats the engine attaches to every result</t>
@@ -667,8 +673,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblLoans" displayName="tblLoans" ref="A1:AI9">
-  <tableColumns count="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblLoans" displayName="tblLoans" ref="A1:AJ9">
+  <tableColumns count="36">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="loan_id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="borrower_reference"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="year_loan_made"/>
@@ -745,6 +751,9 @@
     </tableColumn>
     <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Input_problem">
       <calculatedColumnFormula>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Sample_row">
+      <calculatedColumnFormula>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1126,7 +1135,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AI9"/>
+  <dimension ref="A1:AJ9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1138,10 +1147,10 @@
     <col min="14" max="28" width="12" customWidth="1"/>
     <col min="29" max="29" width="40" customWidth="1"/>
     <col min="30" max="32" width="14" customWidth="1"/>
-    <col min="33" max="35" width="12" customWidth="1"/>
+    <col min="33" max="36" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>9</v>
       </c>
@@ -1247,31 +1256,34 @@
       <c r="AI1" s="5" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ1" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F2" s="7">
         <v>7</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I2" s="7">
         <v>8.2699999999999996E-2</v>
@@ -1371,31 +1383,35 @@
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
       </c>
-    </row>
-    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ2" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F3" s="7">
         <v>7</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I3" s="7">
         <v>0.04</v>
@@ -1495,31 +1511,35 @@
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
       </c>
-    </row>
-    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ3" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F4" s="7">
         <v>7</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I4" s="7">
         <v>4.5199999999999997E-2</v>
@@ -1619,31 +1639,35 @@
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
       </c>
-    </row>
-    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ4" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F5" s="7">
         <v>7</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I5" s="7">
         <v>8.77E-2</v>
@@ -1655,7 +1679,7 @@
         <v>5</v>
       </c>
       <c r="L5" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
@@ -1743,31 +1767,35 @@
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
       </c>
-    </row>
-    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ5" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F6" s="7">
         <v>7</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I6" s="7">
         <v>5.3699999999999998E-2</v>
@@ -1867,28 +1895,32 @@
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
       </c>
-    </row>
-    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ6" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F7" s="7">
         <v>25</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H7" s="7">
         <v>1.0900000000000001</v>
@@ -1991,46 +2023,50 @@
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
       </c>
-    </row>
-    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ7" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="L8" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N8" s="6"/>
       <c r="O8" s="9" t="str">
@@ -2117,31 +2153,35 @@
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
       </c>
-    </row>
-    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ8" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F9" s="7">
         <v>7</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I9" s="7">
         <v>7.0000000000000007E-2</v>
@@ -2240,6 +2280,10 @@
       <c r="AI9" s="9" t="str">
         <f>TRIM(IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_loan_made]])=7,MID(tblLoans[[#This Row],[year_loan_made]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_loan_made]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_loan_made]],4))+1,100)),FALSE))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[year_of_income_being_tested]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(IFERROR(AND(LEN(tblLoans[[#This Row],[year_of_income_being_tested]])=7,MID(tblLoans[[#This Row],[year_of_income_being_tested]],5,1)="-",ISNUMBER(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))),ISNUMBER(VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))),VALUE(RIGHT(tblLoans[[#This Row],[year_of_income_being_tested]],2))=MOD(VALUE(LEFT(tblLoans[[#This Row],[year_of_income_being_tested]],4))+1,100)),FALSE)))),"year label ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[written_agreement]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[terms_in_place_before_lodgment_day]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"}))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[secured_by_registered_mortgage_over_real_property]]&amp;""))={"0","1","f","false","n","no","t","true","y","yes"})))),"true/false/unknown ","")&amp;IF(OR(AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[maximum_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[maximum_term_years]]),OR(tblLoans[[#This Row],[maximum_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[security_coverage_at_first_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]])),AND(ISNUMBER(tblLoans[[#This Row],[security_coverage_at_first_made]]),OR(tblLoans[[#This Row],[security_coverage_at_first_made]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]])),AND(ISNUMBER(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]),OR(tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&lt;0,tblLoans[[#This Row],[interest_rate_for_years_after_year_loan_made]]&gt;1)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]])),AND(ISNUMBER(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]),OR(tblLoans[[#This Row],[amalgamated_loan_unpaid_at_end_of_previous_year]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[remaining_term_years]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]])),AND(ISNUMBER(tblLoans[[#This Row],[remaining_term_years]]),OR(tblLoans[[#This Row],[remaining_term_years]]&lt;0)))),AND(NOT(OR(LOWER(TRIM(tblLoans[[#This Row],[payments_applied_during_the_year]]&amp;""))={"","-","?","n/a","na","unk","unknown"})),OR(NOT(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]])),AND(ISNUMBER(tblLoans[[#This Row],[payments_applied_during_the_year]]),OR(tblLoans[[#This Row],[payments_applied_during_the_year]]&lt;0))))),"number ",""))</f>
         <v/>
+      </c>
+      <c r="AJ9" s="9">
+        <f>IF(SUMPRODUCT((tblLoans[[#This Row],[loan_id]]&amp;""={"L-101","L-102","L-103","L-104","L-105","L-106","L-107","L-108"})*(tblLoans[[#This Row],[year_loan_made]]&amp;""={"2023-24","2022-23","2021-22","2024-25","2019-20","2020-21","2023-24","1996-97"}))&gt;0,1,0)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -2265,214 +2309,214 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B2" s="7">
         <v>5.3699999999999998E-2</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B3" s="7">
         <v>4.5199999999999997E-2</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E3" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="G3" s="7" t="s">
         <v>83</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B4" s="7">
         <v>4.5199999999999997E-2</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B5" s="7">
         <v>4.7699999999999999E-2</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B6" s="7">
         <v>8.2699999999999996E-2</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B7" s="7">
         <v>8.77E-2</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B8" s="7">
         <v>8.3699999999999997E-2</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B9" s="7">
         <v>8.77E-2</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -2494,21 +2538,21 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B1" s="5"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B3" s="12">
         <f>IFERROR(INDEX(tblRates[rate],MATCH(B2,tblRates[year_of_income],0)),"")</f>
@@ -2517,7 +2561,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B4" s="9">
         <f>IFERROR(VALUE(LEFT(B2,4)),"")</f>
@@ -2526,13 +2570,13 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B6" s="5"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B7" s="9">
         <f>COUNTIF(tblLoans[Status],"REVIEWED")</f>
@@ -2541,7 +2585,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B8" s="9">
         <f>COUNTIF(tblLoans[Gate_verdict],"COMPLYING")</f>
@@ -2550,7 +2594,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B9" s="9">
         <f>COUNTIF(tblLoans[Gate_verdict],"NOT_COMPLYING")</f>
@@ -2559,7 +2603,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B10" s="9">
         <f>COUNTIF(tblLoans[MYR_verdict],"MYR_MET")</f>
@@ -2568,7 +2612,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B11" s="9">
         <f>COUNTIF(tblLoans[MYR_verdict],"MYR_SHORT")</f>
@@ -2577,7 +2621,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B12" s="9">
         <f>SUM(tblLoans[Undecided])</f>
@@ -2586,7 +2630,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B13" s="9">
         <f>COUNTIF(tblLoans[MYR_verdict],"REFUSED")</f>
@@ -2595,7 +2639,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B14" s="9">
         <f>COUNTIF(tblLoans[Status],"SKIPPED")</f>
@@ -2604,7 +2648,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B15" s="10">
         <f>SUM(tblLoans[Exposure])</f>
@@ -2661,21 +2705,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B2" s="9" t="str">
         <f>IF(C2=0,"PASS","BLOCKED")</f>
@@ -2692,7 +2736,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B3" s="9" t="str">
         <f>IF(C3=0,"PASS","BLOCKED")</f>
@@ -2709,7 +2753,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B4" s="9" t="str">
         <f>IF(ISNUMBER(Summary!B3),"PASS","BLOCKED")</f>
@@ -2723,7 +2767,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B5" s="9" t="str">
         <f>IF(C5=0,"PASS","REVIEW")</f>
@@ -2740,7 +2784,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B6" s="9" t="str">
         <f>IF(C6=0,"PASS","REVIEW")</f>
@@ -2757,7 +2801,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B7" s="9" t="str">
         <f>IF(C7=0,"PASS","REVIEW")</f>
@@ -2774,7 +2818,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B8" s="9" t="str">
         <f>IF(C8=0,"PASS","NOTE")</f>
@@ -2789,43 +2833,60 @@
         <v>L-106</v>
       </c>
     </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B9" s="9" t="str">
+        <f>IF(C9=0,"PASS","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="C9" s="9">
+        <f>SUM(tblLoans[Sample_row])</f>
+        <v>8</v>
+      </c>
+      <c r="D9" s="9" t="str">
+        <f t="array" ref="D9">IF(C9=0,"",INDEX(tblLoans[loan_id],SUMPRODUCT(MAX((tblLoans[Sample_row]=1)*(ROW(tblLoans[loan_id])-1)))))</f>
+        <v>L-108</v>
+      </c>
+    </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B10" s="13" t="str">
-        <f>IF(COUNTIF(B2:B8,"BLOCKED")&gt;0,"BLOCKED",IF(COUNTIF(B2:B8,"REVIEW")&gt;0,"REVIEW","PASS"))</f>
+        <f>IF(COUNTIF(B2:B9,"BLOCKED")&gt;0,"BLOCKED",IF(COUNTIF(B2:B9,"REVIEW")&gt;0,"REVIEW","PASS"))</f>
         <v>REVIEW</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -2856,82 +2917,82 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B4" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B10" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>